<commit_message>
Hopefully last spreadsheet git commit
</commit_message>
<xml_diff>
--- a/ProductBacklog.xlsx
+++ b/ProductBacklog.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
   <si>
     <t xml:space="preserve">Team:</t>
   </si>
@@ -37,6 +37,9 @@
     <t xml:space="preserve">User Story ID</t>
   </si>
   <si>
+    <t xml:space="preserve">Story # in previous assignment</t>
+  </si>
+  <si>
     <t xml:space="preserve">User Story</t>
   </si>
   <si>
@@ -50,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">Done?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priority: 10 Highest 160 Lowest</t>
   </si>
   <si>
     <t xml:space="preserve">narrow down the hotel listings by price range</t>
@@ -242,23 +248,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
 </styleSheet>
 </file>
 
@@ -439,13 +428,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="56.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="7.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="11.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="56.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="7.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="11.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -455,24 +446,25 @@
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="C1" s="4"/>
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" s="7" customFormat="true" ht="30.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" s="7" customFormat="true" ht="45.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>7</v>
       </c>
       <c r="F3" s="6" t="s">
@@ -481,227 +473,281 @@
       <c r="G3" s="6" t="s">
         <v>9</v>
       </c>
+      <c r="H3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>11</v>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="B5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>11</v>
+      <c r="H5" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="B6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>11</v>
+      <c r="H6" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="B7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>11</v>
+      <c r="H7" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="2" t="n">
+      <c r="B8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>11</v>
+      <c r="H8" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="2" t="n">
+      <c r="B9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="9" t="n">
+      <c r="B10" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="9" t="n">
         <v>70</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="2" t="n">
+      <c r="B11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="2" t="n">
+      <c r="B12" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="G12" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="2" t="n">
+      <c r="B13" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H13" s="2"/>
+      <c r="H13" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="2" t="n">
+      <c r="B14" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="2" t="n">
         <v>110</v>
       </c>
-      <c r="G14" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H14" s="2"/>
+      <c r="H14" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="2" t="n">
+      <c r="B15" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="2" t="n">
+      <c r="B16" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="2" t="n">
         <v>130</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="2" t="n">
+      <c r="B17" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="2" t="n">
         <v>140</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="2" t="n">
+      <c r="B18" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="G18" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C19" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="2" t="n">
+      <c r="B19" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="G19" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G20" s="8"/>
-      <c r="H20" s="2"/>
+      <c r="H20" s="8"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G21" s="8"/>
-      <c r="H21" s="2"/>
+      <c r="H21" s="8"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>